<commit_message>
rebuild the references and composites against the phenotype tree
</commit_message>
<xml_diff>
--- a/04_Figures/F05_classification/c_data/results.xlsx
+++ b/04_Figures/F05_classification/c_data/results.xlsx
@@ -495,7 +495,7 @@
         <v>15</v>
       </c>
       <c r="F2" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -530,7 +530,7 @@
         <v>15</v>
       </c>
       <c r="F3" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G3" t="n">
         <v>200</v>
@@ -548,10 +548,10 @@
         <v>1</v>
       </c>
       <c r="L3" t="n">
-        <v>0.0684821428571428</v>
+        <v>0.0630357142857143</v>
       </c>
       <c r="M3" t="n">
-        <v>0.197675004312679</v>
+        <v>0.191926228301501</v>
       </c>
     </row>
     <row r="4">
@@ -571,7 +571,7 @@
         <v>15</v>
       </c>
       <c r="F4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -606,7 +606,7 @@
         <v>15</v>
       </c>
       <c r="F5" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G5" t="n">
         <v>200</v>
@@ -624,10 +624,10 @@
         <v>1</v>
       </c>
       <c r="L5" t="n">
-        <v>0.0696428571428571</v>
+        <v>0.063125</v>
       </c>
       <c r="M5" t="n">
-        <v>0.206416592006167</v>
+        <v>0.194785083577329</v>
       </c>
     </row>
     <row r="6">
@@ -647,19 +647,19 @@
         <v>15</v>
       </c>
       <c r="F6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>0.0535714285714286</v>
+        <v>0.125</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>0.169651163202309</v>
+        <v>0.369995498067507</v>
       </c>
       <c r="K6"/>
       <c r="L6"/>
@@ -682,28 +682,28 @@
         <v>15</v>
       </c>
       <c r="F7" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G7" t="n">
         <v>200</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0535714285714286</v>
+        <v>0.125</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>0.169651163202309</v>
+        <v>0.369995498067507</v>
       </c>
       <c r="K7" t="n">
-        <v>0.517412935323383</v>
+        <v>0.388059701492537</v>
       </c>
       <c r="L7" t="n">
-        <v>0.154196428571429</v>
+        <v>0.130357142857143</v>
       </c>
       <c r="M7" t="n">
-        <v>0.200399379947737</v>
+        <v>0.184659326226387</v>
       </c>
     </row>
     <row r="8">
@@ -723,19 +723,19 @@
         <v>15</v>
       </c>
       <c r="F8" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>0.607142857142857</v>
+        <v>0.723214285714286</v>
       </c>
       <c r="I8" t="n">
-        <v>0.327304292957517</v>
+        <v>0.433140603759377</v>
       </c>
       <c r="J8" t="n">
-        <v>0.886981421328197</v>
+        <v>1</v>
       </c>
       <c r="K8"/>
       <c r="L8"/>
@@ -758,28 +758,28 @@
         <v>15</v>
       </c>
       <c r="F9" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G9" t="n">
         <v>200</v>
       </c>
       <c r="H9" t="n">
-        <v>0.607142857142857</v>
+        <v>0.723214285714286</v>
       </c>
       <c r="I9" t="n">
-        <v>0.327304292957517</v>
+        <v>0.433140603759377</v>
       </c>
       <c r="J9" t="n">
-        <v>0.886981421328197</v>
+        <v>1</v>
       </c>
       <c r="K9" t="n">
-        <v>0.313432835820896</v>
+        <v>0.149253731343284</v>
       </c>
       <c r="L9" t="n">
-        <v>0.52</v>
+        <v>0.509866071428571</v>
       </c>
       <c r="M9" t="n">
-        <v>0.170882190420093</v>
+        <v>0.181857765842163</v>
       </c>
     </row>
     <row r="10">
@@ -799,19 +799,19 @@
         <v>15</v>
       </c>
       <c r="F10" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>0.410714285714286</v>
+        <v>0.553571428571429</v>
       </c>
       <c r="I10" t="n">
-        <v>0.0949802156730738</v>
+        <v>0.233616372813172</v>
       </c>
       <c r="J10" t="n">
-        <v>0.726448355755498</v>
+        <v>0.873526484329685</v>
       </c>
       <c r="K10"/>
       <c r="L10"/>
@@ -834,28 +834,28 @@
         <v>15</v>
       </c>
       <c r="F11" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G11" t="n">
         <v>200</v>
       </c>
       <c r="H11" t="n">
-        <v>0.410714285714286</v>
+        <v>0.553571428571429</v>
       </c>
       <c r="I11" t="n">
-        <v>0.0949802156730738</v>
+        <v>0.233616372813172</v>
       </c>
       <c r="J11" t="n">
-        <v>0.726448355755498</v>
+        <v>0.873526484329685</v>
       </c>
       <c r="K11" t="n">
-        <v>0.477611940298507</v>
+        <v>0.228855721393035</v>
       </c>
       <c r="L11" t="n">
-        <v>0.377857142857143</v>
+        <v>0.383303571428571</v>
       </c>
       <c r="M11" t="n">
-        <v>0.207341724475913</v>
+        <v>0.208293502413979</v>
       </c>
     </row>
     <row r="12">
@@ -875,7 +875,7 @@
         <v>15</v>
       </c>
       <c r="F12" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -910,7 +910,7 @@
         <v>15</v>
       </c>
       <c r="F13" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G13" t="n">
         <v>200</v>
@@ -928,10 +928,10 @@
         <v>1</v>
       </c>
       <c r="L13" t="n">
-        <v>0.0224107142857143</v>
+        <v>0.02875</v>
       </c>
       <c r="M13" t="n">
-        <v>0.100808785465621</v>
+        <v>0.126911974683316</v>
       </c>
     </row>
     <row r="14">
@@ -951,19 +951,19 @@
         <v>15</v>
       </c>
       <c r="F14" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>0.482142857142857</v>
+        <v>0.410714285714286</v>
       </c>
       <c r="I14" t="n">
-        <v>0.15721293680321</v>
+        <v>0.0862334739795216</v>
       </c>
       <c r="J14" t="n">
-        <v>0.807072777482505</v>
+        <v>0.73519509744905</v>
       </c>
       <c r="K14"/>
       <c r="L14"/>
@@ -986,28 +986,28 @@
         <v>15</v>
       </c>
       <c r="F15" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G15" t="n">
         <v>200</v>
       </c>
       <c r="H15" t="n">
-        <v>0.482142857142857</v>
+        <v>0.410714285714286</v>
       </c>
       <c r="I15" t="n">
-        <v>0.15721293680321</v>
+        <v>0.0862334739795216</v>
       </c>
       <c r="J15" t="n">
-        <v>0.807072777482505</v>
+        <v>0.73519509744905</v>
       </c>
       <c r="K15" t="n">
-        <v>0.393034825870647</v>
+        <v>0.487562189054726</v>
       </c>
       <c r="L15" t="n">
-        <v>0.415089285714286</v>
+        <v>0.405089285714286</v>
       </c>
       <c r="M15" t="n">
-        <v>0.212886505506446</v>
+        <v>0.206870825875968</v>
       </c>
     </row>
     <row r="16">
@@ -1027,19 +1027,19 @@
         <v>15</v>
       </c>
       <c r="F16" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>0.357142857142857</v>
+        <v>0.285714285714286</v>
       </c>
       <c r="I16" t="n">
-        <v>0.037278969659926</v>
+        <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>0.677006744625788</v>
+        <v>0.586111273504665</v>
       </c>
       <c r="K16"/>
       <c r="L16"/>
@@ -1062,28 +1062,28 @@
         <v>15</v>
       </c>
       <c r="F17" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G17" t="n">
         <v>200</v>
       </c>
       <c r="H17" t="n">
-        <v>0.357142857142857</v>
+        <v>0.285714285714286</v>
       </c>
       <c r="I17" t="n">
-        <v>0.037278969659926</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>0.677006744625788</v>
+        <v>0.586111273504665</v>
       </c>
       <c r="K17" t="n">
-        <v>0.383084577114428</v>
+        <v>0.462686567164179</v>
       </c>
       <c r="L17" t="n">
-        <v>0.30875</v>
+        <v>0.312410714285714</v>
       </c>
       <c r="M17" t="n">
-        <v>0.251709301179509</v>
+        <v>0.274051944806005</v>
       </c>
     </row>
     <row r="18">
@@ -1103,7 +1103,7 @@
         <v>15</v>
       </c>
       <c r="F18" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
@@ -1138,7 +1138,7 @@
         <v>15</v>
       </c>
       <c r="F19" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G19" t="n">
         <v>200</v>
@@ -1156,10 +1156,10 @@
         <v>1</v>
       </c>
       <c r="L19" t="n">
-        <v>0.0674107142857143</v>
+        <v>0.0589285714285714</v>
       </c>
       <c r="M19" t="n">
-        <v>0.1857101225098</v>
+        <v>0.173048104873612</v>
       </c>
     </row>
     <row r="20">
@@ -1179,7 +1179,7 @@
         <v>15</v>
       </c>
       <c r="F20" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
@@ -1214,7 +1214,7 @@
         <v>15</v>
       </c>
       <c r="F21" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G21" t="n">
         <v>200</v>
@@ -1232,10 +1232,10 @@
         <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>0.0733928571428571</v>
+        <v>0.0573214285714286</v>
       </c>
       <c r="M21" t="n">
-        <v>0.207429422173081</v>
+        <v>0.177884446682823</v>
       </c>
     </row>
     <row r="22">
@@ -1255,7 +1255,7 @@
         <v>15</v>
       </c>
       <c r="F22" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
@@ -1290,7 +1290,7 @@
         <v>15</v>
       </c>
       <c r="F23" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G23" t="n">
         <v>200</v>
@@ -1308,10 +1308,10 @@
         <v>1</v>
       </c>
       <c r="L23" t="n">
-        <v>0.193839285714286</v>
+        <v>0.190357142857143</v>
       </c>
       <c r="M23" t="n">
-        <v>0.23845508334732</v>
+        <v>0.24348263060434</v>
       </c>
     </row>
     <row r="24">
@@ -1331,19 +1331,19 @@
         <v>15</v>
       </c>
       <c r="F24" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>0.526785714285714</v>
+        <v>0.633928571428571</v>
       </c>
       <c r="I24" t="n">
-        <v>0.248672145078251</v>
+        <v>0.351651393887878</v>
       </c>
       <c r="J24" t="n">
-        <v>0.804899283493177</v>
+        <v>0.916205748969265</v>
       </c>
       <c r="K24"/>
       <c r="L24"/>
@@ -1366,28 +1366,28 @@
         <v>15</v>
       </c>
       <c r="F25" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G25" t="n">
         <v>200</v>
       </c>
       <c r="H25" t="n">
-        <v>0.526785714285714</v>
+        <v>0.633928571428571</v>
       </c>
       <c r="I25" t="n">
-        <v>0.248672145078251</v>
+        <v>0.351651393887878</v>
       </c>
       <c r="J25" t="n">
-        <v>0.804899283493177</v>
+        <v>0.916205748969265</v>
       </c>
       <c r="K25" t="n">
-        <v>0.467661691542289</v>
+        <v>0.263681592039801</v>
       </c>
       <c r="L25" t="n">
-        <v>0.538169642857143</v>
+        <v>0.5153125</v>
       </c>
       <c r="M25" t="n">
-        <v>0.21462743731738</v>
+        <v>0.187873260022492</v>
       </c>
     </row>
     <row r="26">
@@ -1407,19 +1407,19 @@
         <v>15</v>
       </c>
       <c r="F26" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G26" t="n">
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>0.196428571428571</v>
+        <v>0.214285714285714</v>
       </c>
       <c r="I26" t="n">
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>0.433067414378383</v>
+        <v>0.468052601982907</v>
       </c>
       <c r="K26"/>
       <c r="L26"/>
@@ -1442,28 +1442,28 @@
         <v>15</v>
       </c>
       <c r="F27" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G27" t="n">
         <v>200</v>
       </c>
       <c r="H27" t="n">
-        <v>0.196428571428571</v>
+        <v>0.214285714285714</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>0.433067414378383</v>
+        <v>0.468052601982907</v>
       </c>
       <c r="K27" t="n">
-        <v>0.796019900497512</v>
+        <v>0.756218905472637</v>
       </c>
       <c r="L27" t="n">
-        <v>0.381071428571429</v>
+        <v>0.392589285714286</v>
       </c>
       <c r="M27" t="n">
-        <v>0.220742342624846</v>
+        <v>0.224984741076044</v>
       </c>
     </row>
     <row r="28">
@@ -1483,7 +1483,7 @@
         <v>15</v>
       </c>
       <c r="F28" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
@@ -1518,7 +1518,7 @@
         <v>15</v>
       </c>
       <c r="F29" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G29" t="n">
         <v>200</v>
@@ -1536,10 +1536,10 @@
         <v>1</v>
       </c>
       <c r="L29" t="n">
-        <v>0.04625</v>
+        <v>0.0415178571428571</v>
       </c>
       <c r="M29" t="n">
-        <v>0.162110964698251</v>
+        <v>0.157668733367119</v>
       </c>
     </row>
     <row r="30">
@@ -1559,19 +1559,19 @@
         <v>15</v>
       </c>
       <c r="F30" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G30" t="n">
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>0.303571428571429</v>
+        <v>0.196428571428571</v>
       </c>
       <c r="I30" t="n">
-        <v>0.0164791596570672</v>
+        <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>0.59066369748579</v>
+        <v>0.432944132868089</v>
       </c>
       <c r="K30"/>
       <c r="L30"/>
@@ -1594,28 +1594,28 @@
         <v>15</v>
       </c>
       <c r="F31" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G31" t="n">
         <v>200</v>
       </c>
       <c r="H31" t="n">
-        <v>0.303571428571429</v>
+        <v>0.196428571428571</v>
       </c>
       <c r="I31" t="n">
-        <v>0.0164791596570672</v>
+        <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>0.59066369748579</v>
+        <v>0.432944132868089</v>
       </c>
       <c r="K31" t="n">
-        <v>0.761194029850746</v>
+        <v>0.840796019900497</v>
       </c>
       <c r="L31" t="n">
-        <v>0.442321428571429</v>
+        <v>0.430089285714286</v>
       </c>
       <c r="M31" t="n">
-        <v>0.22057001594774</v>
+        <v>0.22882855173496</v>
       </c>
     </row>
     <row r="32">
@@ -1635,19 +1635,19 @@
         <v>15</v>
       </c>
       <c r="F32" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G32" t="n">
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>0.160714285714286</v>
+        <v>0.142857142857143</v>
       </c>
       <c r="I32" t="n">
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>0.3865050288574</v>
+        <v>0.337874925644572</v>
       </c>
       <c r="K32"/>
       <c r="L32"/>
@@ -1670,28 +1670,28 @@
         <v>15</v>
       </c>
       <c r="F33" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G33" t="n">
         <v>200</v>
       </c>
       <c r="H33" t="n">
-        <v>0.160714285714286</v>
+        <v>0.142857142857143</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>0.3865050288574</v>
+        <v>0.337874925644572</v>
       </c>
       <c r="K33" t="n">
-        <v>0.601990049751244</v>
+        <v>0.606965174129353</v>
       </c>
       <c r="L33" t="n">
-        <v>0.308035714285714</v>
+        <v>0.306339285714286</v>
       </c>
       <c r="M33" t="n">
-        <v>0.265798803511816</v>
+        <v>0.271963012755683</v>
       </c>
     </row>
     <row r="34">
@@ -1711,7 +1711,7 @@
         <v>15</v>
       </c>
       <c r="F34" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G34" t="n">
         <v>0</v>
@@ -1746,7 +1746,7 @@
         <v>15</v>
       </c>
       <c r="F35" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G35" t="n">
         <v>200</v>
@@ -1764,10 +1764,10 @@
         <v>1</v>
       </c>
       <c r="L35" t="n">
-        <v>0.0775</v>
+        <v>0.0511607142857143</v>
       </c>
       <c r="M35" t="n">
-        <v>0.206451056585465</v>
+        <v>0.16743521895316</v>
       </c>
     </row>
     <row r="36">
@@ -1787,7 +1787,7 @@
         <v>15</v>
       </c>
       <c r="F36" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G36" t="n">
         <v>0</v>
@@ -1822,7 +1822,7 @@
         <v>15</v>
       </c>
       <c r="F37" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G37" t="n">
         <v>200</v>
@@ -1840,10 +1840,10 @@
         <v>1</v>
       </c>
       <c r="L37" t="n">
-        <v>0.0714285714285714</v>
+        <v>0.0519642857142857</v>
       </c>
       <c r="M37" t="n">
-        <v>0.195926232301198</v>
+        <v>0.176887157549663</v>
       </c>
     </row>
     <row r="38">
@@ -1863,19 +1863,19 @@
         <v>15</v>
       </c>
       <c r="F38" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G38" t="n">
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="I38" t="n">
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>0</v>
+        <v>0.369995498067507</v>
       </c>
       <c r="K38"/>
       <c r="L38"/>
@@ -1898,28 +1898,28 @@
         <v>15</v>
       </c>
       <c r="F39" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G39" t="n">
         <v>200</v>
       </c>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="I39" t="n">
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>0</v>
+        <v>0.369995498067507</v>
       </c>
       <c r="K39" t="n">
-        <v>1</v>
+        <v>0.437810945273632</v>
       </c>
       <c r="L39" t="n">
-        <v>0.166964285714286</v>
+        <v>0.149464285714286</v>
       </c>
       <c r="M39" t="n">
-        <v>0.208814992044325</v>
+        <v>0.19799520465546</v>
       </c>
     </row>
     <row r="40">
@@ -1939,19 +1939,19 @@
         <v>15</v>
       </c>
       <c r="F40" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G40" t="n">
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>0.491071428571429</v>
+        <v>0.267857142857143</v>
       </c>
       <c r="I40" t="n">
-        <v>0.209440757256154</v>
+        <v>0.0262179060489883</v>
       </c>
       <c r="J40" t="n">
-        <v>0.772702099886704</v>
+        <v>0.509496379665297</v>
       </c>
       <c r="K40"/>
       <c r="L40"/>
@@ -1974,28 +1974,28 @@
         <v>15</v>
       </c>
       <c r="F41" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G41" t="n">
         <v>200</v>
       </c>
       <c r="H41" t="n">
-        <v>0.491071428571429</v>
+        <v>0.267857142857143</v>
       </c>
       <c r="I41" t="n">
-        <v>0.209440757256154</v>
+        <v>0.0262179060489883</v>
       </c>
       <c r="J41" t="n">
-        <v>0.772702099886704</v>
+        <v>0.509496379665297</v>
       </c>
       <c r="K41" t="n">
-        <v>0.557213930348259</v>
+        <v>0.885572139303483</v>
       </c>
       <c r="L41" t="n">
-        <v>0.524732142857143</v>
+        <v>0.515625</v>
       </c>
       <c r="M41" t="n">
-        <v>0.19122586445159</v>
+        <v>0.20398164846116</v>
       </c>
     </row>
     <row r="42">
@@ -2015,19 +2015,19 @@
         <v>15</v>
       </c>
       <c r="F42" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G42" t="n">
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>0.482142857142857</v>
+        <v>0.428571428571429</v>
       </c>
       <c r="I42" t="n">
-        <v>0.144016946322232</v>
+        <v>0.105622257708171</v>
       </c>
       <c r="J42" t="n">
-        <v>0.820268767963482</v>
+        <v>0.751520599434686</v>
       </c>
       <c r="K42"/>
       <c r="L42"/>
@@ -2050,28 +2050,28 @@
         <v>15</v>
       </c>
       <c r="F43" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G43" t="n">
         <v>200</v>
       </c>
       <c r="H43" t="n">
-        <v>0.482142857142857</v>
+        <v>0.428571428571429</v>
       </c>
       <c r="I43" t="n">
-        <v>0.144016946322232</v>
+        <v>0.105622257708171</v>
       </c>
       <c r="J43" t="n">
-        <v>0.820268767963482</v>
+        <v>0.751520599434686</v>
       </c>
       <c r="K43" t="n">
-        <v>0.333333333333333</v>
+        <v>0.398009950248756</v>
       </c>
       <c r="L43" t="n">
-        <v>0.365535714285714</v>
+        <v>0.366160714285714</v>
       </c>
       <c r="M43" t="n">
-        <v>0.231537465075451</v>
+        <v>0.219625657378727</v>
       </c>
     </row>
     <row r="44">
@@ -2091,7 +2091,7 @@
         <v>15</v>
       </c>
       <c r="F44" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G44" t="n">
         <v>0</v>
@@ -2126,7 +2126,7 @@
         <v>15</v>
       </c>
       <c r="F45" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G45" t="n">
         <v>200</v>
@@ -2144,10 +2144,10 @@
         <v>1</v>
       </c>
       <c r="L45" t="n">
-        <v>0.039375</v>
+        <v>0.023125</v>
       </c>
       <c r="M45" t="n">
-        <v>0.153834953742725</v>
+        <v>0.112281041550031</v>
       </c>
     </row>
     <row r="46">
@@ -2167,19 +2167,19 @@
         <v>15</v>
       </c>
       <c r="F46" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G46" t="n">
         <v>0</v>
       </c>
       <c r="H46" t="n">
-        <v>0.339285714285714</v>
+        <v>0.321428571428571</v>
       </c>
       <c r="I46" t="n">
-        <v>0.0360861846501504</v>
+        <v>0.0229797039788519</v>
       </c>
       <c r="J46" t="n">
-        <v>0.642485243921278</v>
+        <v>0.619877438878291</v>
       </c>
       <c r="K46"/>
       <c r="L46"/>
@@ -2202,28 +2202,28 @@
         <v>15</v>
       </c>
       <c r="F47" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G47" t="n">
         <v>200</v>
       </c>
       <c r="H47" t="n">
-        <v>0.339285714285714</v>
+        <v>0.321428571428571</v>
       </c>
       <c r="I47" t="n">
-        <v>0.0360861846501504</v>
+        <v>0.0229797039788519</v>
       </c>
       <c r="J47" t="n">
-        <v>0.642485243921278</v>
+        <v>0.619877438878291</v>
       </c>
       <c r="K47" t="n">
-        <v>0.691542288557214</v>
+        <v>0.646766169154229</v>
       </c>
       <c r="L47" t="n">
-        <v>0.421875</v>
+        <v>0.414375</v>
       </c>
       <c r="M47" t="n">
-        <v>0.213644931344176</v>
+        <v>0.211851282116214</v>
       </c>
     </row>
     <row r="48">
@@ -2243,19 +2243,19 @@
         <v>15</v>
       </c>
       <c r="F48" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G48" t="n">
         <v>0</v>
       </c>
       <c r="H48" t="n">
-        <v>0.267857142857143</v>
+        <v>0.446428571428571</v>
       </c>
       <c r="I48" t="n">
-        <v>0</v>
+        <v>0.13069450138736</v>
       </c>
       <c r="J48" t="n">
-        <v>0.537991032177125</v>
+        <v>0.762162641469783</v>
       </c>
       <c r="K48"/>
       <c r="L48"/>
@@ -2278,28 +2278,28 @@
         <v>15</v>
       </c>
       <c r="F49" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G49" t="n">
         <v>200</v>
       </c>
       <c r="H49" t="n">
-        <v>0.267857142857143</v>
+        <v>0.446428571428571</v>
       </c>
       <c r="I49" t="n">
-        <v>0</v>
+        <v>0.13069450138736</v>
       </c>
       <c r="J49" t="n">
-        <v>0.537991032177125</v>
+        <v>0.762162641469783</v>
       </c>
       <c r="K49" t="n">
-        <v>0.502487562189055</v>
+        <v>0.258706467661692</v>
       </c>
       <c r="L49" t="n">
-        <v>0.3175</v>
+        <v>0.304196428571429</v>
       </c>
       <c r="M49" t="n">
-        <v>0.261068925571557</v>
+        <v>0.24079543705373</v>
       </c>
     </row>
     <row r="50">
@@ -2319,7 +2319,7 @@
         <v>15</v>
       </c>
       <c r="F50" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G50" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
         <v>15</v>
       </c>
       <c r="F51" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G51" t="n">
         <v>200</v>
@@ -2372,10 +2372,10 @@
         <v>1</v>
       </c>
       <c r="L51" t="n">
-        <v>0.0566071428571429</v>
+        <v>0.0495535714285714</v>
       </c>
       <c r="M51" t="n">
-        <v>0.181553615951543</v>
+        <v>0.167442492198123</v>
       </c>
     </row>
     <row r="52">
@@ -2395,7 +2395,7 @@
         <v>15</v>
       </c>
       <c r="F52" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G52" t="n">
         <v>0</v>
@@ -2430,7 +2430,7 @@
         <v>15</v>
       </c>
       <c r="F53" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G53" t="n">
         <v>200</v>
@@ -2448,10 +2448,10 @@
         <v>1</v>
       </c>
       <c r="L53" t="n">
-        <v>0.0625892857142857</v>
+        <v>0.0554464285714286</v>
       </c>
       <c r="M53" t="n">
-        <v>0.191542519437959</v>
+        <v>0.180485057842753</v>
       </c>
     </row>
     <row r="54">
@@ -2471,19 +2471,19 @@
         <v>15</v>
       </c>
       <c r="F54" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G54" t="n">
         <v>0</v>
       </c>
       <c r="H54" t="n">
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="I54" t="n">
         <v>0</v>
       </c>
       <c r="J54" t="n">
-        <v>0</v>
+        <v>0.312079431647071</v>
       </c>
       <c r="K54"/>
       <c r="L54"/>
@@ -2506,28 +2506,28 @@
         <v>15</v>
       </c>
       <c r="F55" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G55" t="n">
         <v>200</v>
       </c>
       <c r="H55" t="n">
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="I55" t="n">
         <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>0</v>
+        <v>0.312079431647071</v>
       </c>
       <c r="K55" t="n">
-        <v>1</v>
+        <v>0.3681592039801</v>
       </c>
       <c r="L55" t="n">
-        <v>0.129642857142857</v>
+        <v>0.121607142857143</v>
       </c>
       <c r="M55" t="n">
-        <v>0.195034700782402</v>
+        <v>0.188212376933318</v>
       </c>
     </row>
     <row r="56">
@@ -2547,19 +2547,19 @@
         <v>15</v>
       </c>
       <c r="F56" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G56" t="n">
         <v>0</v>
       </c>
       <c r="H56" t="n">
-        <v>0.276785714285714</v>
+        <v>0.446428571428571</v>
       </c>
       <c r="I56" t="n">
-        <v>0.0439676352772868</v>
+        <v>0.164797900113296</v>
       </c>
       <c r="J56" t="n">
-        <v>0.509603793294142</v>
+        <v>0.728059242743846</v>
       </c>
       <c r="K56"/>
       <c r="L56"/>
@@ -2582,28 +2582,28 @@
         <v>15</v>
       </c>
       <c r="F57" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G57" t="n">
         <v>200</v>
       </c>
       <c r="H57" t="n">
-        <v>0.276785714285714</v>
+        <v>0.446428571428571</v>
       </c>
       <c r="I57" t="n">
-        <v>0.0439676352772868</v>
+        <v>0.164797900113296</v>
       </c>
       <c r="J57" t="n">
-        <v>0.509603793294142</v>
+        <v>0.728059242743846</v>
       </c>
       <c r="K57" t="n">
-        <v>0.970149253731343</v>
+        <v>0.616915422885572</v>
       </c>
       <c r="L57" t="n">
-        <v>0.506294642857143</v>
+        <v>0.510982142857143</v>
       </c>
       <c r="M57" t="n">
-        <v>0.173796067612305</v>
+        <v>0.177386841729617</v>
       </c>
     </row>
     <row r="58">
@@ -2623,19 +2623,19 @@
         <v>15</v>
       </c>
       <c r="F58" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G58" t="n">
         <v>0</v>
       </c>
       <c r="H58" t="n">
-        <v>0.464285714285714</v>
+        <v>0.410714285714286</v>
       </c>
       <c r="I58" t="n">
-        <v>0.142875483057025</v>
+        <v>0.077891616708458</v>
       </c>
       <c r="J58" t="n">
-        <v>0.785695945514403</v>
+        <v>0.743536954720113</v>
       </c>
       <c r="K58"/>
       <c r="L58"/>
@@ -2658,28 +2658,28 @@
         <v>15</v>
       </c>
       <c r="F59" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G59" t="n">
         <v>200</v>
       </c>
       <c r="H59" t="n">
-        <v>0.464285714285714</v>
+        <v>0.410714285714286</v>
       </c>
       <c r="I59" t="n">
-        <v>0.142875483057025</v>
+        <v>0.077891616708458</v>
       </c>
       <c r="J59" t="n">
-        <v>0.785695945514403</v>
+        <v>0.743536954720113</v>
       </c>
       <c r="K59" t="n">
-        <v>0.313432835820896</v>
+        <v>0.383084577114428</v>
       </c>
       <c r="L59" t="n">
-        <v>0.3475</v>
+        <v>0.343571428571429</v>
       </c>
       <c r="M59" t="n">
-        <v>0.218600669468398</v>
+        <v>0.218023749740075</v>
       </c>
     </row>
     <row r="60">
@@ -2699,7 +2699,7 @@
         <v>15</v>
       </c>
       <c r="F60" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G60" t="n">
         <v>0</v>
@@ -2734,7 +2734,7 @@
         <v>15</v>
       </c>
       <c r="F61" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G61" t="n">
         <v>200</v>
@@ -2752,10 +2752,10 @@
         <v>1</v>
       </c>
       <c r="L61" t="n">
-        <v>0.0316964285714286</v>
+        <v>0.0271428571428571</v>
       </c>
       <c r="M61" t="n">
-        <v>0.143945930534148</v>
+        <v>0.136030820646376</v>
       </c>
     </row>
     <row r="62">
@@ -2775,19 +2775,19 @@
         <v>15</v>
       </c>
       <c r="F62" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G62" t="n">
         <v>0</v>
       </c>
       <c r="H62" t="n">
-        <v>0.392857142857143</v>
+        <v>0.464285714285714</v>
       </c>
       <c r="I62" t="n">
-        <v>0.0501901257460894</v>
+        <v>0.112215014215032</v>
       </c>
       <c r="J62" t="n">
-        <v>0.735524159968196</v>
+        <v>0.816356414356396</v>
       </c>
       <c r="K62"/>
       <c r="L62"/>
@@ -2810,28 +2810,28 @@
         <v>15</v>
       </c>
       <c r="F63" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G63" t="n">
         <v>200</v>
       </c>
       <c r="H63" t="n">
-        <v>0.392857142857143</v>
+        <v>0.464285714285714</v>
       </c>
       <c r="I63" t="n">
-        <v>0.0501901257460894</v>
+        <v>0.112215014215032</v>
       </c>
       <c r="J63" t="n">
-        <v>0.735524159968196</v>
+        <v>0.816356414356396</v>
       </c>
       <c r="K63" t="n">
-        <v>0.512437810945274</v>
+        <v>0.318407960199005</v>
       </c>
       <c r="L63" t="n">
-        <v>0.392232142857143</v>
+        <v>0.357589285714286</v>
       </c>
       <c r="M63" t="n">
-        <v>0.22419206161625</v>
+        <v>0.229420627702577</v>
       </c>
     </row>
     <row r="64">
@@ -2851,19 +2851,19 @@
         <v>15</v>
       </c>
       <c r="F64" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G64" t="n">
         <v>0</v>
       </c>
       <c r="H64" t="n">
-        <v>0.375</v>
+        <v>0.357142857142857</v>
       </c>
       <c r="I64" t="n">
-        <v>0.0462330699664537</v>
+        <v>0.0403943037600185</v>
       </c>
       <c r="J64" t="n">
-        <v>0.703766930033546</v>
+        <v>0.673891410525696</v>
       </c>
       <c r="K64"/>
       <c r="L64"/>
@@ -2886,28 +2886,28 @@
         <v>15</v>
       </c>
       <c r="F65" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G65" t="n">
         <v>200</v>
       </c>
       <c r="H65" t="n">
-        <v>0.375</v>
+        <v>0.357142857142857</v>
       </c>
       <c r="I65" t="n">
-        <v>0.0462330699664537</v>
+        <v>0.0403943037600185</v>
       </c>
       <c r="J65" t="n">
-        <v>0.703766930033546</v>
+        <v>0.673891410525696</v>
       </c>
       <c r="K65" t="n">
-        <v>0.333333333333333</v>
+        <v>0.338308457711443</v>
       </c>
       <c r="L65" t="n">
-        <v>0.286071428571429</v>
+        <v>0.287589285714286</v>
       </c>
       <c r="M65" t="n">
-        <v>0.249390087723598</v>
+        <v>0.258274990779136</v>
       </c>
     </row>
     <row r="66">
@@ -2927,7 +2927,7 @@
         <v>14</v>
       </c>
       <c r="F66" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G66" t="n">
         <v>0</v>
@@ -2962,7 +2962,7 @@
         <v>14</v>
       </c>
       <c r="F67" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G67" t="n">
         <v>200</v>
@@ -2980,10 +2980,10 @@
         <v>1</v>
       </c>
       <c r="L67" t="n">
-        <v>0.075625</v>
+        <v>0.0515625</v>
       </c>
       <c r="M67" t="n">
-        <v>0.209443336910788</v>
+        <v>0.167044921220645</v>
       </c>
     </row>
     <row r="68">
@@ -3003,7 +3003,7 @@
         <v>14</v>
       </c>
       <c r="F68" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G68" t="n">
         <v>0</v>
@@ -3038,7 +3038,7 @@
         <v>14</v>
       </c>
       <c r="F69" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G69" t="n">
         <v>200</v>
@@ -3056,10 +3056,10 @@
         <v>1</v>
       </c>
       <c r="L69" t="n">
-        <v>0.0701041666666666</v>
+        <v>0.0492708333333333</v>
       </c>
       <c r="M69" t="n">
-        <v>0.203086972452924</v>
+        <v>0.174631420451172</v>
       </c>
     </row>
     <row r="70">
@@ -3079,19 +3079,19 @@
         <v>14</v>
       </c>
       <c r="F70" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G70" t="n">
         <v>0</v>
       </c>
       <c r="H70" t="n">
-        <v>0.104166666666667</v>
+        <v>0</v>
       </c>
       <c r="I70" t="n">
         <v>0</v>
       </c>
       <c r="J70" t="n">
-        <v>0.312372804231433</v>
+        <v>0</v>
       </c>
       <c r="K70"/>
       <c r="L70"/>
@@ -3114,28 +3114,28 @@
         <v>14</v>
       </c>
       <c r="F71" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G71" t="n">
         <v>200</v>
       </c>
       <c r="H71" t="n">
-        <v>0.104166666666667</v>
+        <v>0</v>
       </c>
       <c r="I71" t="n">
         <v>0</v>
       </c>
       <c r="J71" t="n">
-        <v>0.312372804231433</v>
+        <v>0</v>
       </c>
       <c r="K71" t="n">
-        <v>0.3681592039801</v>
+        <v>1</v>
       </c>
       <c r="L71" t="n">
-        <v>0.115833333333333</v>
+        <v>0.108958333333333</v>
       </c>
       <c r="M71" t="n">
-        <v>0.19343325047604</v>
+        <v>0.185008219406345</v>
       </c>
     </row>
     <row r="72">
@@ -3155,19 +3155,19 @@
         <v>14</v>
       </c>
       <c r="F72" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G72" t="n">
         <v>0</v>
       </c>
       <c r="H72" t="n">
-        <v>0.895833333333333</v>
+        <v>0.208333333333333</v>
       </c>
       <c r="I72" t="n">
-        <v>0.722320592265192</v>
+        <v>0</v>
       </c>
       <c r="J72" t="n">
-        <v>1</v>
+        <v>0.437245657092439</v>
       </c>
       <c r="K72"/>
       <c r="L72"/>
@@ -3190,28 +3190,28 @@
         <v>14</v>
       </c>
       <c r="F73" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G73" t="n">
         <v>200</v>
       </c>
       <c r="H73" t="n">
-        <v>0.895833333333333</v>
+        <v>0.208333333333333</v>
       </c>
       <c r="I73" t="n">
-        <v>0.722320592265192</v>
+        <v>0</v>
       </c>
       <c r="J73" t="n">
-        <v>1</v>
+        <v>0.437245657092439</v>
       </c>
       <c r="K73" t="n">
-        <v>0.0447761194029851</v>
+        <v>0.950248756218905</v>
       </c>
       <c r="L73" t="n">
-        <v>0.49359375</v>
+        <v>0.51703125</v>
       </c>
       <c r="M73" t="n">
-        <v>0.192741725172994</v>
+        <v>0.2174291037597</v>
       </c>
     </row>
     <row r="74">
@@ -3231,19 +3231,19 @@
         <v>14</v>
       </c>
       <c r="F74" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G74" t="n">
         <v>0</v>
       </c>
       <c r="H74" t="n">
-        <v>0.5</v>
+        <v>0.458333333333333</v>
       </c>
       <c r="I74" t="n">
-        <v>0.123478920716696</v>
+        <v>0.101027399641709</v>
       </c>
       <c r="J74" t="n">
-        <v>0.876521079283304</v>
+        <v>0.815639267024957</v>
       </c>
       <c r="K74"/>
       <c r="L74"/>
@@ -3266,28 +3266,28 @@
         <v>14</v>
       </c>
       <c r="F75" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G75" t="n">
         <v>200</v>
       </c>
       <c r="H75" t="n">
-        <v>0.5</v>
+        <v>0.458333333333333</v>
       </c>
       <c r="I75" t="n">
-        <v>0.123478920716696</v>
+        <v>0.101027399641709</v>
       </c>
       <c r="J75" t="n">
-        <v>0.876521079283304</v>
+        <v>0.815639267024957</v>
       </c>
       <c r="K75" t="n">
-        <v>0.218905472636816</v>
+        <v>0.258706467661692</v>
       </c>
       <c r="L75" t="n">
-        <v>0.31875</v>
+        <v>0.321666666666667</v>
       </c>
       <c r="M75" t="n">
-        <v>0.203653467402439</v>
+        <v>0.203949265513279</v>
       </c>
     </row>
     <row r="76">
@@ -3307,7 +3307,7 @@
         <v>14</v>
       </c>
       <c r="F76" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G76" t="n">
         <v>0</v>
@@ -3342,7 +3342,7 @@
         <v>14</v>
       </c>
       <c r="F77" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G77" t="n">
         <v>200</v>
@@ -3360,10 +3360,10 @@
         <v>1</v>
       </c>
       <c r="L77" t="n">
-        <v>0.00239583333333333</v>
+        <v>0.0319791666666667</v>
       </c>
       <c r="M77" t="n">
-        <v>0.020375785910038</v>
+        <v>0.13292962430867</v>
       </c>
     </row>
     <row r="78">
@@ -3383,19 +3383,19 @@
         <v>14</v>
       </c>
       <c r="F78" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G78" t="n">
         <v>0</v>
       </c>
       <c r="H78" t="n">
-        <v>0.25</v>
+        <v>0.291666666666667</v>
       </c>
       <c r="I78" t="n">
         <v>0</v>
       </c>
       <c r="J78" t="n">
-        <v>0.551798290501113</v>
+        <v>0.607351466771162</v>
       </c>
       <c r="K78"/>
       <c r="L78"/>
@@ -3418,28 +3418,28 @@
         <v>14</v>
       </c>
       <c r="F79" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G79" t="n">
         <v>200</v>
       </c>
       <c r="H79" t="n">
-        <v>0.25</v>
+        <v>0.291666666666667</v>
       </c>
       <c r="I79" t="n">
         <v>0</v>
       </c>
       <c r="J79" t="n">
-        <v>0.551798290501113</v>
+        <v>0.607351466771162</v>
       </c>
       <c r="K79" t="n">
-        <v>0.796019900497512</v>
+        <v>0.671641791044776</v>
       </c>
       <c r="L79" t="n">
-        <v>0.402395833333333</v>
+        <v>0.366979166666667</v>
       </c>
       <c r="M79" t="n">
-        <v>0.220267256477767</v>
+        <v>0.208078544994611</v>
       </c>
     </row>
     <row r="80">
@@ -3459,19 +3459,19 @@
         <v>14</v>
       </c>
       <c r="F80" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G80" t="n">
         <v>0</v>
       </c>
       <c r="H80" t="n">
-        <v>0.0416666666666667</v>
+        <v>0.291666666666667</v>
       </c>
       <c r="I80" t="n">
         <v>0</v>
       </c>
       <c r="J80" t="n">
-        <v>0.138294194204506</v>
+        <v>0.601871468483091</v>
       </c>
       <c r="K80"/>
       <c r="L80"/>
@@ -3494,28 +3494,28 @@
         <v>14</v>
       </c>
       <c r="F81" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G81" t="n">
         <v>200</v>
       </c>
       <c r="H81" t="n">
-        <v>0.0416666666666667</v>
+        <v>0.291666666666667</v>
       </c>
       <c r="I81" t="n">
         <v>0</v>
       </c>
       <c r="J81" t="n">
-        <v>0.138294194204506</v>
+        <v>0.601871468483091</v>
       </c>
       <c r="K81" t="n">
-        <v>0.890547263681592</v>
+        <v>0.402985074626866</v>
       </c>
       <c r="L81" t="n">
-        <v>0.318125</v>
+        <v>0.301145833333333</v>
       </c>
       <c r="M81" t="n">
-        <v>0.262758191732864</v>
+        <v>0.269341801147164</v>
       </c>
     </row>
     <row r="82">
@@ -3535,7 +3535,7 @@
         <v>14</v>
       </c>
       <c r="F82" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G82" t="n">
         <v>0</v>
@@ -3570,7 +3570,7 @@
         <v>14</v>
       </c>
       <c r="F83" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G83" t="n">
         <v>200</v>
@@ -3588,10 +3588,10 @@
         <v>1</v>
       </c>
       <c r="L83" t="n">
-        <v>0.0864583333333333</v>
+        <v>0.078125</v>
       </c>
       <c r="M83" t="n">
-        <v>0.205601328806589</v>
+        <v>0.199277095077576</v>
       </c>
     </row>
     <row r="84">
@@ -3611,7 +3611,7 @@
         <v>14</v>
       </c>
       <c r="F84" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G84" t="n">
         <v>0</v>
@@ -3646,7 +3646,7 @@
         <v>14</v>
       </c>
       <c r="F85" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G85" t="n">
         <v>200</v>
@@ -3664,10 +3664,10 @@
         <v>1</v>
       </c>
       <c r="L85" t="n">
-        <v>0.08375</v>
+        <v>0.069375</v>
       </c>
       <c r="M85" t="n">
-        <v>0.207104415628062</v>
+        <v>0.187797665265799</v>
       </c>
     </row>
     <row r="86">
@@ -3687,7 +3687,7 @@
         <v>14</v>
       </c>
       <c r="F86" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G86" t="n">
         <v>0</v>
@@ -3722,7 +3722,7 @@
         <v>14</v>
       </c>
       <c r="F87" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G87" t="n">
         <v>200</v>
@@ -3740,10 +3740,10 @@
         <v>1</v>
       </c>
       <c r="L87" t="n">
-        <v>0.152083333333333</v>
+        <v>0.14125</v>
       </c>
       <c r="M87" t="n">
-        <v>0.221859873482685</v>
+        <v>0.211266619676689</v>
       </c>
     </row>
     <row r="88">
@@ -3763,19 +3763,19 @@
         <v>14</v>
       </c>
       <c r="F88" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G88" t="n">
         <v>0</v>
       </c>
       <c r="H88" t="n">
-        <v>0.71875</v>
+        <v>0.270833333333333</v>
       </c>
       <c r="I88" t="n">
-        <v>0.432297612212229</v>
+        <v>0.0282805233732971</v>
       </c>
       <c r="J88" t="n">
-        <v>1</v>
+        <v>0.51338614329337</v>
       </c>
       <c r="K88"/>
       <c r="L88"/>
@@ -3798,28 +3798,28 @@
         <v>14</v>
       </c>
       <c r="F89" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G89" t="n">
         <v>200</v>
       </c>
       <c r="H89" t="n">
-        <v>0.71875</v>
+        <v>0.270833333333333</v>
       </c>
       <c r="I89" t="n">
-        <v>0.432297612212229</v>
+        <v>0.0282805233732971</v>
       </c>
       <c r="J89" t="n">
-        <v>1</v>
+        <v>0.51338614329337</v>
       </c>
       <c r="K89" t="n">
-        <v>0.159203980099502</v>
+        <v>0.895522388059702</v>
       </c>
       <c r="L89" t="n">
-        <v>0.50359375</v>
+        <v>0.525416666666667</v>
       </c>
       <c r="M89" t="n">
-        <v>0.198856912912421</v>
+        <v>0.213298353333767</v>
       </c>
     </row>
     <row r="90">
@@ -3839,19 +3839,19 @@
         <v>14</v>
       </c>
       <c r="F90" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G90" t="n">
         <v>0</v>
       </c>
       <c r="H90" t="n">
-        <v>0.125</v>
+        <v>0.1875</v>
       </c>
       <c r="I90" t="n">
         <v>0</v>
       </c>
       <c r="J90" t="n">
-        <v>0.341065720072343</v>
+        <v>0.456411092588118</v>
       </c>
       <c r="K90"/>
       <c r="L90"/>
@@ -3874,28 +3874,28 @@
         <v>14</v>
       </c>
       <c r="F91" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G91" t="n">
         <v>200</v>
       </c>
       <c r="H91" t="n">
-        <v>0.125</v>
+        <v>0.1875</v>
       </c>
       <c r="I91" t="n">
         <v>0</v>
       </c>
       <c r="J91" t="n">
-        <v>0.341065720072343</v>
+        <v>0.456411092588118</v>
       </c>
       <c r="K91" t="n">
-        <v>0.830845771144279</v>
+        <v>0.72636815920398</v>
       </c>
       <c r="L91" t="n">
-        <v>0.340729166666667</v>
+        <v>0.342604166666667</v>
       </c>
       <c r="M91" t="n">
-        <v>0.217831009112221</v>
+        <v>0.208570818369027</v>
       </c>
     </row>
     <row r="92">
@@ -3915,7 +3915,7 @@
         <v>14</v>
       </c>
       <c r="F92" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G92" t="n">
         <v>0</v>
@@ -3950,7 +3950,7 @@
         <v>14</v>
       </c>
       <c r="F93" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G93" t="n">
         <v>200</v>
@@ -3968,10 +3968,10 @@
         <v>1</v>
       </c>
       <c r="L93" t="n">
-        <v>0.00604166666666664</v>
+        <v>0.0398958333333333</v>
       </c>
       <c r="M93" t="n">
-        <v>0.0527373096343631</v>
+        <v>0.163346022511147</v>
       </c>
     </row>
     <row r="94">
@@ -3991,19 +3991,19 @@
         <v>14</v>
       </c>
       <c r="F94" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G94" t="n">
         <v>0</v>
       </c>
       <c r="H94" t="n">
-        <v>0.229166666666667</v>
+        <v>0.270833333333333</v>
       </c>
       <c r="I94" t="n">
         <v>0</v>
       </c>
       <c r="J94" t="n">
-        <v>0.553338730186194</v>
+        <v>0.60025312738578</v>
       </c>
       <c r="K94"/>
       <c r="L94"/>
@@ -4026,28 +4026,28 @@
         <v>14</v>
       </c>
       <c r="F95" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G95" t="n">
         <v>200</v>
       </c>
       <c r="H95" t="n">
-        <v>0.229166666666667</v>
+        <v>0.270833333333333</v>
       </c>
       <c r="I95" t="n">
         <v>0</v>
       </c>
       <c r="J95" t="n">
-        <v>0.553338730186194</v>
+        <v>0.60025312738578</v>
       </c>
       <c r="K95" t="n">
-        <v>0.791044776119403</v>
+        <v>0.736318407960199</v>
       </c>
       <c r="L95" t="n">
-        <v>0.411770833333333</v>
+        <v>0.415104166666667</v>
       </c>
       <c r="M95" t="n">
-        <v>0.221121117712336</v>
+        <v>0.228761228645274</v>
       </c>
     </row>
     <row r="96">
@@ -4067,19 +4067,19 @@
         <v>14</v>
       </c>
       <c r="F96" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G96" t="n">
         <v>0</v>
       </c>
       <c r="H96" t="n">
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="I96" t="n">
         <v>0</v>
       </c>
       <c r="J96" t="n">
-        <v>0</v>
+        <v>0.319238547712681</v>
       </c>
       <c r="K96"/>
       <c r="L96"/>
@@ -4102,28 +4102,28 @@
         <v>14</v>
       </c>
       <c r="F97" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G97" t="n">
         <v>200</v>
       </c>
       <c r="H97" t="n">
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="I97" t="n">
         <v>0</v>
       </c>
       <c r="J97" t="n">
-        <v>0</v>
+        <v>0.319238547712681</v>
       </c>
       <c r="K97" t="n">
-        <v>1</v>
+        <v>0.671641791044776</v>
       </c>
       <c r="L97" t="n">
-        <v>0.325208333333333</v>
+        <v>0.314270833333333</v>
       </c>
       <c r="M97" t="n">
-        <v>0.273033279330559</v>
+        <v>0.274220838450523</v>
       </c>
     </row>
     <row r="98">
@@ -4143,7 +4143,7 @@
         <v>14</v>
       </c>
       <c r="F98" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="G98" t="n">
         <v>0</v>
@@ -4178,7 +4178,7 @@
         <v>14</v>
       </c>
       <c r="F99" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="G99" t="n">
         <v>200</v>
@@ -4196,10 +4196,10 @@
         <v>1</v>
       </c>
       <c r="L99" t="n">
-        <v>0.0634375</v>
+        <v>0.075</v>
       </c>
       <c r="M99" t="n">
-        <v>0.178816678096809</v>
+        <v>0.205455415343636</v>
       </c>
     </row>
     <row r="100">
@@ -4219,7 +4219,7 @@
         <v>14</v>
       </c>
       <c r="F100" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="G100" t="n">
         <v>0</v>
@@ -4254,7 +4254,7 @@
         <v>14</v>
       </c>
       <c r="F101" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="G101" t="n">
         <v>200</v>
@@ -4272,10 +4272,10 @@
         <v>1</v>
       </c>
       <c r="L101" t="n">
-        <v>0.0611458333333334</v>
+        <v>0.0780208333333333</v>
       </c>
       <c r="M101" t="n">
-        <v>0.187343801260896</v>
+        <v>0.210623897696129</v>
       </c>
     </row>
     <row r="102">
@@ -4295,19 +4295,19 @@
         <v>14</v>
       </c>
       <c r="F102" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="G102" t="n">
         <v>0</v>
       </c>
       <c r="H102" t="n">
-        <v>0</v>
+        <v>0.166666666666667</v>
       </c>
       <c r="I102" t="n">
         <v>0</v>
       </c>
       <c r="J102" t="n">
-        <v>0</v>
+        <v>0.404158501418271</v>
       </c>
       <c r="K102"/>
       <c r="L102"/>
@@ -4330,28 +4330,28 @@
         <v>14</v>
       </c>
       <c r="F103" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="G103" t="n">
         <v>200</v>
       </c>
       <c r="H103" t="n">
-        <v>0</v>
+        <v>0.166666666666667</v>
       </c>
       <c r="I103" t="n">
         <v>0</v>
       </c>
       <c r="J103" t="n">
-        <v>0</v>
+        <v>0.404158501418271</v>
       </c>
       <c r="K103" t="n">
-        <v>1</v>
+        <v>0.348258706467662</v>
       </c>
       <c r="L103" t="n">
-        <v>0.170416666666667</v>
+        <v>0.164375</v>
       </c>
       <c r="M103" t="n">
-        <v>0.229064428237211</v>
+        <v>0.21942610082072</v>
       </c>
     </row>
     <row r="104">
@@ -4371,19 +4371,19 @@
         <v>14</v>
       </c>
       <c r="F104" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="G104" t="n">
         <v>0</v>
       </c>
       <c r="H104" t="n">
-        <v>0.354166666666667</v>
+        <v>0.229166666666667</v>
       </c>
       <c r="I104" t="n">
-        <v>0.0435015062465005</v>
+        <v>0</v>
       </c>
       <c r="J104" t="n">
-        <v>0.664831827086833</v>
+        <v>0.48833526969636</v>
       </c>
       <c r="K104"/>
       <c r="L104"/>
@@ -4406,28 +4406,28 @@
         <v>14</v>
       </c>
       <c r="F105" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="G105" t="n">
         <v>200</v>
       </c>
       <c r="H105" t="n">
-        <v>0.354166666666667</v>
+        <v>0.229166666666667</v>
       </c>
       <c r="I105" t="n">
-        <v>0.0435015062465005</v>
+        <v>0</v>
       </c>
       <c r="J105" t="n">
-        <v>0.664831827086833</v>
+        <v>0.48833526969636</v>
       </c>
       <c r="K105" t="n">
-        <v>0.432835820895522</v>
+        <v>0.651741293532338</v>
       </c>
       <c r="L105" t="n">
-        <v>0.333645833333333</v>
+        <v>0.3359375</v>
       </c>
       <c r="M105" t="n">
-        <v>0.209767649462179</v>
+        <v>0.211388171579236</v>
       </c>
     </row>
     <row r="106">
@@ -4447,7 +4447,7 @@
         <v>14</v>
       </c>
       <c r="F106" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="G106" t="n">
         <v>0</v>
@@ -4482,7 +4482,7 @@
         <v>14</v>
       </c>
       <c r="F107" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="G107" t="n">
         <v>200</v>
@@ -4500,10 +4500,10 @@
         <v>1</v>
       </c>
       <c r="L107" t="n">
-        <v>0.00239583333333334</v>
+        <v>0.00322916666666666</v>
       </c>
       <c r="M107" t="n">
-        <v>0.0219226817414016</v>
+        <v>0.025071218700313</v>
       </c>
     </row>
     <row r="108">
@@ -4523,19 +4523,19 @@
         <v>14</v>
       </c>
       <c r="F108" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="G108" t="n">
         <v>0</v>
       </c>
       <c r="H108" t="n">
-        <v>0.4375</v>
+        <v>0.416666666666667</v>
       </c>
       <c r="I108" t="n">
-        <v>0.0900629437137719</v>
+        <v>0.0879707139504487</v>
       </c>
       <c r="J108" t="n">
-        <v>0.784937056286228</v>
+        <v>0.745362619382885</v>
       </c>
       <c r="K108"/>
       <c r="L108"/>
@@ -4558,28 +4558,28 @@
         <v>14</v>
       </c>
       <c r="F109" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="G109" t="n">
         <v>200</v>
       </c>
       <c r="H109" t="n">
-        <v>0.4375</v>
+        <v>0.416666666666667</v>
       </c>
       <c r="I109" t="n">
-        <v>0.0900629437137719</v>
+        <v>0.0879707139504487</v>
       </c>
       <c r="J109" t="n">
-        <v>0.784937056286228</v>
+        <v>0.745362619382885</v>
       </c>
       <c r="K109" t="n">
-        <v>0.497512437810945</v>
+        <v>0.487562189054726</v>
       </c>
       <c r="L109" t="n">
-        <v>0.434791666666667</v>
+        <v>0.418958333333333</v>
       </c>
       <c r="M109" t="n">
-        <v>0.219381566149401</v>
+        <v>0.220160414810613</v>
       </c>
     </row>
     <row r="110">
@@ -4599,19 +4599,19 @@
         <v>14</v>
       </c>
       <c r="F110" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="G110" t="n">
         <v>0</v>
       </c>
       <c r="H110" t="n">
-        <v>0.395833333333333</v>
+        <v>0.0833333333333333</v>
       </c>
       <c r="I110" t="n">
-        <v>0.0664135392808862</v>
+        <v>0</v>
       </c>
       <c r="J110" t="n">
-        <v>0.72525312738578</v>
+        <v>0.254635630756703</v>
       </c>
       <c r="K110"/>
       <c r="L110"/>
@@ -4634,28 +4634,28 @@
         <v>14</v>
       </c>
       <c r="F111" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="G111" t="n">
         <v>200</v>
       </c>
       <c r="H111" t="n">
-        <v>0.395833333333333</v>
+        <v>0.0833333333333333</v>
       </c>
       <c r="I111" t="n">
-        <v>0.0664135392808862</v>
+        <v>0</v>
       </c>
       <c r="J111" t="n">
-        <v>0.72525312738578</v>
+        <v>0.254635630756703</v>
       </c>
       <c r="K111" t="n">
-        <v>0.378109452736318</v>
+        <v>0.835820895522388</v>
       </c>
       <c r="L111" t="n">
-        <v>0.334166666666667</v>
+        <v>0.340729166666667</v>
       </c>
       <c r="M111" t="n">
-        <v>0.256424296581201</v>
+        <v>0.262427517012814</v>
       </c>
     </row>
     <row r="112">
@@ -12158,47 +12158,6 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" t="n">
-        <v>14</v>
-      </c>
-      <c r="F2" t="n">
-        <v>13</v>
-      </c>
-      <c r="G2" t="n">
-        <v>200</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0.895833333333333</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0.722320592265192</v>
-      </c>
-      <c r="J2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0.0447761194029851</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0.49359375</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0.192741725172994</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>